<commit_message>
worked on profile completion error
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5208DB75-C2E6-44CB-BFED-3CD8B7CAA1BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85C5A12-46F8-403C-8FA7-3343F0E6AC80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Email</t>
   </si>
@@ -57,7 +58,70 @@
     <t>Test@123</t>
   </si>
   <si>
-    <t>abhijithlok6535</t>
+    <t>AboutMe</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Pincode</t>
+  </si>
+  <si>
+    <t>HouseNo</t>
+  </si>
+  <si>
+    <t>District</t>
+  </si>
+  <si>
+    <t>CompanyName</t>
+  </si>
+  <si>
+    <t>PassportNo</t>
+  </si>
+  <si>
+    <t>DocNo</t>
+  </si>
+  <si>
+    <t>FbUrl</t>
+  </si>
+  <si>
+    <t>LiUrl</t>
+  </si>
+  <si>
+    <t>InstaUrl</t>
+  </si>
+  <si>
+    <t>Automation QA Engineer with 3+ years experience</t>
+  </si>
+  <si>
+    <t>Flat 12B, Palm Residency</t>
+  </si>
+  <si>
+    <t>TC-45/123</t>
+  </si>
+  <si>
+    <t>Thiruvananthapuram</t>
+  </si>
+  <si>
+    <t>N1234567</t>
+  </si>
+  <si>
+    <t>EID987654</t>
+  </si>
+  <si>
+    <t>https://facebook.com/testuser1</t>
+  </si>
+  <si>
+    <t>https://linkedin.com/in/testuser1</t>
+  </si>
+  <si>
+    <t>https://instagram.com/testuser1</t>
+  </si>
+  <si>
+    <t>Appa Kadai Restaurant - 16th Street - Dubai - United Arab Emirates</t>
+  </si>
+  <si>
+    <t>abhijithlok5822</t>
   </si>
 </sst>
 </file>
@@ -110,7 +174,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -120,6 +184,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -470,7 +537,7 @@
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>6</v>
@@ -495,4 +562,98 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D9E7038-0FBD-4392-A991-C80E0C2D61C0}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="9.21875" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="28.21875" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" customWidth="1"/>
+    <col min="8" max="8" width="16.88671875" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="30.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="4">
+        <v>695003</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
profileCompletion approval added working on Flaky
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC6D2BE-56AD-4D46-A2BA-F74BC5F81989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE75ECB-67A4-4F16-9B81-93CF4F4C7DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4356" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -121,7 +121,7 @@
     <t>Appa Kadai Restaurant - 16th Street - Dubai - United Arab Emirates</t>
   </si>
   <si>
-    <t>abhijithlok5824</t>
+    <t>asp7855</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Profile Completion fixed flakiness
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CA9725-9AA0-4394-95BE-5800D588389F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D131528-4CD7-4994-98D8-A5093EEB6CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
@@ -121,7 +121,7 @@
     <t>Appa Kadai Restaurant - 16th Street - Dubai - United Arab Emirates</t>
   </si>
   <si>
-    <t>asp7859</t>
+    <t>asp1795</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
admin page table details fetching
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D131528-4CD7-4994-98D8-A5093EEB6CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D537E4FB-B433-4987-BCDB-F2B62F1BCF41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
+    <workbookView xWindow="30915" yWindow="2880" windowWidth="21600" windowHeight="11235" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -46,15 +46,9 @@
     <t>Password</t>
   </si>
   <si>
-    <t>Abhijith</t>
-  </si>
-  <si>
     <t>S</t>
   </si>
   <si>
-    <t>Suresh</t>
-  </si>
-  <si>
     <t>Test@123</t>
   </si>
   <si>
@@ -121,7 +115,13 @@
     <t>Appa Kadai Restaurant - 16th Street - Dubai - United Arab Emirates</t>
   </si>
   <si>
-    <t>asp1795</t>
+    <t>Sumesh</t>
+  </si>
+  <si>
+    <t>Anoop</t>
+  </si>
+  <si>
+    <t>asp468</t>
   </si>
 </sst>
 </file>
@@ -507,11 +507,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.88671875" customWidth="1"/>
-    <col min="2" max="2" width="26.21875" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
     <col min="4" max="4" width="28.109375" customWidth="1"/>
-    <col min="5" max="5" width="22.77734375" customWidth="1"/>
-    <col min="6" max="6" width="27.21875" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" customWidth="1"/>
+    <col min="6" max="6" width="27.33203125" customWidth="1"/>
     <col min="7" max="7" width="25.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -540,19 +540,19 @@
         <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="2">
+        <v>9876544213</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2">
-        <v>9876543210</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -571,10 +571,10 @@
   <cols>
     <col min="1" max="1" width="24.33203125" customWidth="1"/>
     <col min="2" max="2" width="14.109375" customWidth="1"/>
-    <col min="3" max="3" width="9.21875" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" customWidth="1"/>
     <col min="4" max="4" width="11.109375" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="28.21875" customWidth="1"/>
+    <col min="6" max="6" width="28.33203125" customWidth="1"/>
     <col min="7" max="7" width="16.109375" customWidth="1"/>
     <col min="8" max="8" width="16.88671875" customWidth="1"/>
     <col min="9" max="9" width="15.44140625" customWidth="1"/>
@@ -584,72 +584,72 @@
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C2" s="4">
         <v>695003</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed flakiness and added LKO ID identical and added new test cases
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D537E4FB-B433-4987-BCDB-F2B62F1BCF41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2D64B40-4D8F-4D65-BDE2-496C4FAF5254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30915" yWindow="2880" windowWidth="21600" windowHeight="11235" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -115,13 +115,13 @@
     <t>Appa Kadai Restaurant - 16th Street - Dubai - United Arab Emirates</t>
   </si>
   <si>
-    <t>Sumesh</t>
-  </si>
-  <si>
-    <t>Anoop</t>
-  </si>
-  <si>
-    <t>asp468</t>
+    <t>asp441</t>
+  </si>
+  <si>
+    <t>Akhil</t>
+  </si>
+  <si>
+    <t>Satheesh</t>
   </si>
 </sst>
 </file>
@@ -537,7 +537,7 @@
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>30</v>
@@ -546,7 +546,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E2" s="2">
         <v>9876544213</v>

</xml_diff>

<commit_message>
Completed new two test cases
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2D64B40-4D8F-4D65-BDE2-496C4FAF5254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2567C329-3B81-4E68-8F7C-29FF1A1F01E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="37">
   <si>
     <t>Email</t>
   </si>
@@ -115,13 +117,28 @@
     <t>Appa Kadai Restaurant - 16th Street - Dubai - United Arab Emirates</t>
   </si>
   <si>
-    <t>asp441</t>
-  </si>
-  <si>
     <t>Akhil</t>
   </si>
   <si>
     <t>Satheesh</t>
+  </si>
+  <si>
+    <t>I am Video Creator settled in Dubai and I am an Entrepreneur also</t>
+  </si>
+  <si>
+    <t>Apartment Number 18J diera Dubai</t>
+  </si>
+  <si>
+    <t>Business Description</t>
+  </si>
+  <si>
+    <t>Founder of Tech Matters</t>
+  </si>
+  <si>
+    <t>asp8557</t>
+  </si>
+  <si>
+    <t>abhi729</t>
   </si>
 </sst>
 </file>
@@ -537,16 +554,16 @@
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E2" s="2">
         <v>9876544213</v>
@@ -656,4 +673,156 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42C82F4E-57FE-403C-925A-C5D640C5A8A3}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.5546875" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" customWidth="1"/>
+    <col min="6" max="6" width="24.21875" customWidth="1"/>
+    <col min="7" max="7" width="20.88671875" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="20.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="4">
+        <v>695003</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D314F62-1879-4ED5-8572-3B057AB5D839}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.109375" customWidth="1"/>
+    <col min="2" max="2" width="19.21875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="18.21875" customWidth="1"/>
+    <col min="5" max="5" width="41.33203125" customWidth="1"/>
+    <col min="6" max="6" width="28.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2">
+        <v>9876544213</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{C1B411A8-4885-4922-89B9-C24705997E81}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added student profile and admin reject
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB1FCBCB-49E3-4198-87F5-37D9A345FAAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED5AEA2-8925-413F-9C72-9958E13E60A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
@@ -152,9 +152,6 @@
     <t>InstituteName</t>
   </si>
   <si>
-    <t xml:space="preserve"> Dubai College - Dubai - United Arab Emirates</t>
-  </si>
-  <si>
     <t>CourseName</t>
   </si>
   <si>
@@ -164,7 +161,10 @@
     <t xml:space="preserve">Studying at Dubai College </t>
   </si>
   <si>
-    <t>asp819</t>
+    <t>Dubai College</t>
+  </si>
+  <si>
+    <t>asp827</t>
   </si>
 </sst>
 </file>
@@ -739,7 +739,7 @@
         <v>39</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>14</v>
@@ -759,7 +759,7 @@
     </row>
     <row r="2" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>20</v>
@@ -774,10 +774,10 @@
         <v>22</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
completed all 15 testcases and optimized flakiness
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{584C6438-FF1F-4966-BF50-973B143E9A7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E041FC08-3B72-47F6-846D-8EA85C2541E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -158,13 +158,13 @@
     <t>Dubai College</t>
   </si>
   <si>
-    <t>asp816</t>
-  </si>
-  <si>
-    <t>asp831</t>
-  </si>
-  <si>
-    <t>abhi750</t>
+    <t>abhijith753</t>
+  </si>
+  <si>
+    <t>arya832</t>
+  </si>
+  <si>
+    <t>adithyan818</t>
   </si>
 </sst>
 </file>
@@ -580,7 +580,7 @@
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>29</v>
@@ -926,7 +926,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
added validation to resubmit and reject profiles, driver.quit active,changed sheet name
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E041FC08-3B72-47F6-846D-8EA85C2541E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F9E129-9B15-4443-A293-BA6529667482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet6" sheetId="6" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId5"/>
-    <sheet name="Sheet5" sheetId="5" r:id="rId6"/>
+    <sheet name="Employee" sheetId="1" r:id="rId1"/>
+    <sheet name="EmployeeProfile" sheetId="2" r:id="rId2"/>
+    <sheet name="StudentProfile" sheetId="6" r:id="rId3"/>
+    <sheet name="EmployerProfile" sheetId="4" r:id="rId4"/>
+    <sheet name="Employer" sheetId="3" r:id="rId5"/>
+    <sheet name="Student" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -140,9 +140,6 @@
     <t>Sidharth</t>
   </si>
   <si>
-    <t>Aswin</t>
-  </si>
-  <si>
     <t>InstituteName</t>
   </si>
   <si>
@@ -158,13 +155,16 @@
     <t>Dubai College</t>
   </si>
   <si>
-    <t>abhijith753</t>
-  </si>
-  <si>
-    <t>arya832</t>
-  </si>
-  <si>
-    <t>adithyan818</t>
+    <t>abhijith754</t>
+  </si>
+  <si>
+    <t>Ajay</t>
+  </si>
+  <si>
+    <t>sam856</t>
+  </si>
+  <si>
+    <t>adithyan821</t>
   </si>
 </sst>
 </file>
@@ -580,7 +580,7 @@
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>29</v>
@@ -736,10 +736,10 @@
         <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>14</v>
@@ -759,7 +759,7 @@
     </row>
     <row r="2" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>20</v>
@@ -774,10 +774,10 @@
         <v>22</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>23</v>
@@ -990,7 +990,7 @@
         <v>43</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Added new test cases 16,17,18 with validation
</commit_message>
<xml_diff>
--- a/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
+++ b/Loka_KeralamOnline_QA-main/src/test/resources/testdata/registrationData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DUK\Downloads\Loka_KeralamOnline_QA-main\Loka_KeralamOnline_QA-main\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F9E129-9B15-4443-A293-BA6529667482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F753BDA1-1854-4006-BF90-364E7381E71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{1CEF1BEB-5E8D-4E58-9A66-459A1AB0894F}"/>
   </bookViews>
   <sheets>
     <sheet name="Employee" sheetId="1" r:id="rId1"/>
@@ -155,16 +155,16 @@
     <t>Dubai College</t>
   </si>
   <si>
-    <t>abhijith754</t>
-  </si>
-  <si>
     <t>Ajay</t>
   </si>
   <si>
-    <t>sam856</t>
-  </si>
-  <si>
-    <t>adithyan821</t>
+    <t>abhijith755</t>
+  </si>
+  <si>
+    <t>sam857</t>
+  </si>
+  <si>
+    <t>adithyan823</t>
   </si>
 </sst>
 </file>
@@ -580,7 +580,7 @@
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>29</v>
@@ -990,7 +990,7 @@
         <v>43</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>6</v>

</xml_diff>